<commit_message>
Align Paul Smart Start story from Excel to UI
</commit_message>
<xml_diff>
--- a/personetics-demo-data.xlsx
+++ b/personetics-demo-data.xlsx
@@ -469,7 +469,7 @@
         <v>Smart Start Account Holder</v>
       </c>
       <c r="C3" t="str">
-        <v>First debit card issued and activated for youth savings</v>
+        <v>Parents deposit pocket money into Paul's Smart Start Account</v>
       </c>
       <c r="D3">
         <v>11</v>
@@ -484,7 +484,7 @@
         <v>Motivation &amp; Goal Achievement</v>
       </c>
       <c r="H3" t="str">
-        <v>Paul receives a Smart Start Account from BOI and his parents deposit EUR20 pocket money. With a goal to save EUR100 for GAA equipment by his birthday, Paul learns the power of consistent saving.</v>
+        <v>Paul is 11, loves sport, and regularly spends on GAA equipment. When his parents lodge €20 into his Smart Start Account, BOI Buddy nudges him toward a €100 birthday savings goal.</v>
       </c>
       <c r="I3" t="str">
         <v>Engagement Lift, Financial Health, Primacy</v>
@@ -1416,10 +1416,10 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Parents deposit EUR20 pocket money - savings goal opportunity</v>
+        <v>Parents deposit pocket money into Paul's Smart Start Account</v>
       </c>
       <c r="F7" t="str">
-        <v>Hey Paul! EUR20 has gone into your account. If you put EUR5 into your Smart Start Money Pot each week, you could have EUR100 by your birthday - that's a lot of GAA gear! If you reach this savings goal, you can earn points to redeem vouchers.</v>
+        <v>Hey Paul! €20 has gone into your account. If you put €5 into your Smart Start Money Pot each week, you could have €100 by your birthday - that's a lot of GAA gear! If you reach this savings goal, you can earn points to redeem vouchers.</v>
       </c>
       <c r="G7" t="str">
         <v>chatbot</v>
@@ -1431,7 +1431,7 @@
         <v>goals_trackers</v>
       </c>
       <c r="J7" t="str">
-        <v>Paul starts his Smart Start Money Pot and begins working toward his EUR100 birthday goal.</v>
+        <v>Paul can see he is already on his way to hitting his €100 birthday goal for new GAA gear.</v>
       </c>
       <c r="K7" t="str">
         <v>Goal tracker adoption increases youth engagement and repeat deposits</v>
@@ -1457,7 +1457,7 @@
         <v>Weekly pocket money habit forming - consistent savings behaviour detected</v>
       </c>
       <c r="F8" t="str">
-        <v>You are one week into your savings plan. Another EUR5 moved into your Money Pot today, so you are already building momentum toward your birthday target.</v>
+        <v>You are one week into your savings plan. Another €5 moved into your Money Pot today, so you are already building momentum toward your birthday target.</v>
       </c>
       <c r="G8" t="str">
         <v>in_app</v>
@@ -1495,7 +1495,7 @@
         <v>Birthday target projection updated - goal remains on track</v>
       </c>
       <c r="F9" t="str">
-        <v>At your current pace, you are still on track to reach EUR100 by your birthday. Keep going and you will be ready for new GAA gear right on time.</v>
+        <v>At your current pace, you are still on track to reach €100 by your birthday. Keep going and you will be ready for new GAA gear right on time.</v>
       </c>
       <c r="G9" t="str">
         <v>push</v>
@@ -1533,7 +1533,7 @@
         <v>Reward threshold approaching - loyalty incentive available</v>
       </c>
       <c r="F10" t="str">
-        <v>You are close to your EUR100 goal. One more good week of saving could unlock reward points that can be redeemed for vouchers.</v>
+        <v>You are close to your €100 goal. One more good week of saving could unlock reward points that can be redeemed for vouchers.</v>
       </c>
       <c r="G10" t="str">
         <v>in_app</v>
@@ -1571,7 +1571,7 @@
         <v>Savings goal achieved - celebration and follow-on habit opportunity</v>
       </c>
       <c r="F11" t="str">
-        <v>You did it, Paul. Your Smart Start Money Pot has reached EUR100 in time for your birthday. Keep the habit going and choose your next savings goal.</v>
+        <v>You did it, Paul. Your Smart Start Money Pot has reached €100 in time for your birthday. Keep the habit going and choose your next savings goal.</v>
       </c>
       <c r="G11" t="str">
         <v>in_app</v>
@@ -1583,7 +1583,7 @@
         <v>goals_trackers</v>
       </c>
       <c r="J11" t="str">
-        <v>Paul reaches his EUR100 goal and feels proud that his saving habit paid off.</v>
+        <v>Paul reaches his €100 goal and feels proud that his saving habit paid off.</v>
       </c>
       <c r="K11" t="str">
         <v>Goal completion improves retention and creates momentum for the next savings objective</v>

</xml_diff>